<commit_message>
dynamic analysis in c++ added: not complete
</commit_message>
<xml_diff>
--- a/Trebuchet/WIPPER_TREBUCHET/WIPPERS_BRAINS.xlsx
+++ b/Trebuchet/WIPPER_TREBUCHET/WIPPERS_BRAINS.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\4aida\OneDrive\Documents\GitHub\Design_II_Group6\Trebuchet\WIPPER_TREBUCHET\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFB25BE4-D717-4DB5-8320-F03949D1B446}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A72CCF89-F1EF-4B2A-9D13-0D6ED46A20EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B1667E68-D567-4D9D-8078-E1F59153EB2C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{B1667E68-D567-4D9D-8078-E1F59153EB2C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Ball weight g</t>
   </si>
@@ -51,9 +50,6 @@
     <t>~kinetic</t>
   </si>
   <si>
-    <t>~ max dist m</t>
-  </si>
-  <si>
     <t>~optimal launch angle deg</t>
   </si>
   <si>
@@ -61,13 +57,38 @@
   </si>
   <si>
     <t>height G-ARM</t>
+  </si>
+  <si>
+    <t>Relistic kenetic</t>
+  </si>
+  <si>
+    <t>efficency</t>
+  </si>
+  <si>
+    <t>relistic dist F</t>
+  </si>
+  <si>
+    <t>relistic dist M</t>
+  </si>
+  <si>
+    <t>~ max dist M</t>
+  </si>
+  <si>
+    <t>Relistic launch angle</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -84,7 +105,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -92,15 +113,239 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -432,79 +677,133 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6724248A-62A3-4482-9A35-E5086BE9D667}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.453125" customWidth="1"/>
     <col min="2" max="2" width="11.54296875" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="3" max="3" width="13.90625" customWidth="1"/>
     <col min="4" max="4" width="23.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="10">
+        <v>2.3E-2</v>
+      </c>
+      <c r="B2" s="17">
+        <v>1.675</v>
+      </c>
+      <c r="C2" s="16">
+        <f>A4*9.81*B2</f>
+        <v>14.049146250000002</v>
+      </c>
+      <c r="D2" s="14">
+        <f>DEGREES(ASIN(1/(SQRT(2+((2*9.891*B4)/(C4^2))))))</f>
+        <v>44.554723439812747</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>2.3E-2</v>
-      </c>
-      <c r="B2">
-        <v>1.6</v>
-      </c>
-      <c r="C2">
-        <f>A5*9.81*B2</f>
-        <v>13.420080000000002</v>
-      </c>
-      <c r="D2">
-        <f>DEGREES(ASIN(1/(SQRT(2+((2*9.891*B4)/(C4^2))))))</f>
-        <v>44.522442837796945</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="C3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="11">
+        <v>0.85499999999999998</v>
+      </c>
+      <c r="B4" s="11">
+        <v>1.95</v>
+      </c>
+      <c r="C4" s="11">
+        <f>SQRT((C2*2)/A2)</f>
+        <v>34.952323117417357</v>
+      </c>
+      <c r="D4" s="15">
+        <f>((C4*COS(RADIANS(D2)))/9.81)*((C4*SIN(RADIANS(D2)))+(SQRT(((C4*SIN(RADIANS(D2)))^2)+(2*9.81*B4))))</f>
+        <v>126.46757512811377</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="7"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="7"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="D6" s="4">
+        <f>DEGREES(ASIN(1/(SQRT(2+((2*9.891*B4)/(C8^2))))))</f>
+        <v>43.297308482277941</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="7"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4">
-        <v>0.28499999999999998</v>
-      </c>
-      <c r="B4">
-        <v>2</v>
-      </c>
-      <c r="C4">
-        <f>SQRT((C2*2)/A2)</f>
-        <v>34.160847153735368</v>
-      </c>
-      <c r="D4">
-        <f>((C4*COS(RADIANS(D2)))/9.81)*((C4*SIN(RADIANS(D2)))+(SQRT(((C4*SIN(RADIANS(D2)))^2)+(2*9.81*B4))))</f>
-        <v>120.93998468682148</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5">
-        <f>A4*3</f>
-        <v>0.85499999999999998</v>
+      <c r="D7" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="7"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="3">
+        <f>C4*C6</f>
+        <v>17.476161558708679</v>
+      </c>
+      <c r="D8" s="4">
+        <f>((C8*COS(RADIANS(D2)))/9.81)*((C8*SIN(RADIANS(D2)))+(SQRT(((C8*SIN(RADIANS(D2)))^2)+(2*9.81*B4))))</f>
+        <v>32.997795866177142</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="7"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="7"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="6">
+        <f>3.28084*D8</f>
+        <v>108.26048858958862</v>
       </c>
     </row>
   </sheetData>

</xml_diff>